<commit_message>
Atualiza dashboard de obras (2026-05-07 10:07:15)
</commit_message>
<xml_diff>
--- a/doc/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/doc/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEBF2523-B246-4AA1-AD38-80CDB183820F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDC3DEE-9F23-4662-862F-278B02A0DDE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="121">
   <si>
     <t>Obra</t>
   </si>
@@ -397,6 +397,9 @@
   </si>
   <si>
     <t>CT LAGEADO MONTANTE</t>
+  </si>
+  <si>
+    <t>concuido</t>
   </si>
 </sst>
 </file>
@@ -7286,7 +7289,9 @@
       <c r="V145" s="6"/>
       <c r="W145" s="6"/>
       <c r="X145" s="6"/>
-      <c r="Y145" s="6"/>
+      <c r="Y145" s="6">
+        <v>42</v>
+      </c>
       <c r="Z145" s="6"/>
       <c r="AA145" s="6"/>
       <c r="AB145" s="6"/>
@@ -7700,7 +7705,7 @@
       <c r="AE156" s="6"/>
       <c r="AF156" s="6"/>
       <c r="AG156" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="157" spans="2:33" x14ac:dyDescent="0.3">
@@ -9051,6 +9056,9 @@
       <c r="D192" t="s">
         <v>6</v>
       </c>
+      <c r="F192" s="5">
+        <v>78.19</v>
+      </c>
       <c r="L192" s="6"/>
       <c r="M192" s="6"/>
       <c r="N192" s="6"/>
@@ -9064,7 +9072,9 @@
       <c r="V192" s="6"/>
       <c r="W192" s="6"/>
       <c r="X192" s="6"/>
-      <c r="Y192" s="6"/>
+      <c r="Y192" s="6">
+        <v>78.19</v>
+      </c>
       <c r="Z192" s="6"/>
       <c r="AA192" s="6"/>
       <c r="AB192" s="6"/>

</xml_diff>

<commit_message>
Atualiza dashboard (JSONs) - 2026-05-13 10:39
</commit_message>
<xml_diff>
--- a/doc/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/doc/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDC3DEE-9F23-4662-862F-278B02A0DDE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F5E3A9A-5019-4D99-8281-814FC022FA8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE_DASH_EXTENSAO" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="121">
   <si>
     <t>Obra</t>
   </si>
@@ -9057,7 +9057,7 @@
         <v>6</v>
       </c>
       <c r="F192" s="5">
-        <v>78.19</v>
+        <v>158.69999999999999</v>
       </c>
       <c r="L192" s="6"/>
       <c r="M192" s="6"/>
@@ -9073,7 +9073,8 @@
       <c r="W192" s="6"/>
       <c r="X192" s="6"/>
       <c r="Y192" s="6">
-        <v>78.19</v>
+        <f>78.19+80.53</f>
+        <v>158.72</v>
       </c>
       <c r="Z192" s="6"/>
       <c r="AA192" s="6"/>
@@ -9490,6 +9491,9 @@
       <c r="AD204" s="6"/>
       <c r="AE204" s="6"/>
       <c r="AF204" s="6"/>
+      <c r="AG204" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="205" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B205" t="s">
@@ -9525,6 +9529,9 @@
       <c r="AD205" s="6"/>
       <c r="AE205" s="6"/>
       <c r="AF205" s="6"/>
+      <c r="AG205" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="206" spans="2:33" x14ac:dyDescent="0.3">
       <c r="B206" s="5" t="s">

</xml_diff>

<commit_message>
Atualiza dashboard obras 2026-05-19 10:09 (-03:00)
</commit_message>
<xml_diff>
--- a/doc/BASE_DASH_EXTENSAO_POWERBI.xlsx
+++ b/doc/BASE_DASH_EXTENSAO_POWERBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCA6F4DA-0E96-4337-9D01-E8E0A6C3B1EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3201084-D6CB-45F5-AA24-265FB3B68E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9061,7 +9061,7 @@
         <v>6</v>
       </c>
       <c r="F192" s="5">
-        <v>158.69999999999999</v>
+        <v>268.02</v>
       </c>
       <c r="L192" s="6"/>
       <c r="M192" s="6"/>
@@ -9077,8 +9077,7 @@
       <c r="W192" s="6"/>
       <c r="X192" s="6"/>
       <c r="Y192" s="6">
-        <f>78.19+80.53</f>
-        <v>158.72</v>
+        <v>268.02</v>
       </c>
       <c r="Z192" s="6"/>
       <c r="AA192" s="6"/>

</xml_diff>